<commit_message>
AB#3822 feat: add student GR number generation feature with new API.
</commit_message>
<xml_diff>
--- a/public/templates/Employee_import_attendance.xlsx
+++ b/public/templates/Employee_import_attendance.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025\Shikshamitra-FE\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBC61F8-68DD-476D-98F7-A35B9D6E69BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97307F60-5FE9-42DB-A949-4248D40977E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11360" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -47,10 +48,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -76,8 +85,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,8 +429,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="16.3984375" customWidth="1"/>
@@ -426,43 +438,30 @@
     <col min="7" max="7" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="E1" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
AB#3822 feat: add student GR number generation feature with new API. (#638)
Co-authored-by: raj <rajbaku222@gmail.com>
</commit_message>
<xml_diff>
--- a/public/templates/Employee_import_attendance.xlsx
+++ b/public/templates/Employee_import_attendance.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2025\Shikshamitra-FE\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBC61F8-68DD-476D-98F7-A35B9D6E69BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97307F60-5FE9-42DB-A949-4248D40977E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11360" yWindow="-21710" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -47,10 +48,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -76,8 +85,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -417,8 +429,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="16.3984375" customWidth="1"/>
@@ -426,43 +438,30 @@
     <col min="7" max="7" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="6" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="7" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:7" ht="15.6" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="E1" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>